<commit_message>
Add column-control block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (6):
- blocks/column-control/_column-control.json
- component-definition.json
- tools/importer/import-merkle-now.bundle.js
- tools/importer/reports/en/merkle-now.report.json
- tools/importer/reports/import-merkle-now.report.xlsx
- tools/importer/transformers/merkle-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-merkle-now.report.xlsx
+++ b/tools/importer/reports/import-merkle-now.report.xlsx
@@ -64,7 +64,7 @@
     <t>en/merkle-now.report.json</t>
   </si>
   <si>
-    <t>["column-control","content-filter"]</t>
+    <t>["column-control"]</t>
   </si>
   <si>
     <t>en/merkle-now</t>
@@ -73,7 +73,7 @@
     <t>merkle-now</t>
   </si>
   <si>
-    <t>2026-09-17T04:56:33.967Z</t>
+    <t>2026-09-17T05:53:46.674Z</t>
   </si>
   <si>
     <t>Merkle Now: Thought Leadership, Culture &amp; Resources</t>

</xml_diff>

<commit_message>
Rename column-control → columns-control for JCR/UE compatibility
md2jcr only exports a block as a multi-column container when its name
starts with "Columns" (splitColumns checks startsWith('columns')), and
Universal Editor resolves the columns resourceType model by that name.
The prior "Column Control" name produced empty columns in JCR and the
"reading 'modelId'" error in UE.

Rename the block (folder, files, CSS classes, JS, model id/title, section
filter, importer parser + scripts, page-templates) to columns-control /
"Columns Control". The Layout select (classes field) is preserved via
template.model, so the layout-* ratio variants still apply. Regenerated
the aggregated component JSON and re-imported merkle-now.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-merkle-now.report.xlsx
+++ b/tools/importer/reports/import-merkle-now.report.xlsx
@@ -64,7 +64,7 @@
     <t>en/merkle-now.report.json</t>
   </si>
   <si>
-    <t>["column-control"]</t>
+    <t>["columns-control"]</t>
   </si>
   <si>
     <t>en/merkle-now</t>
@@ -73,7 +73,7 @@
     <t>merkle-now</t>
   </si>
   <si>
-    <t>2026-09-17T05:53:46.674Z</t>
+    <t>2026-09-17T06:39:57.072Z</t>
   </si>
   <si>
     <t>Merkle Now: Thought Leadership, Culture &amp; Resources</t>

</xml_diff>

<commit_message>
Extend core Columns with ratio layouts; remove columns-control
Fold the ratio-layout capability into the core Columns block and delete
the separate columns-control block.

- Columns model gains a "Layout" select: Equal (default) plus 75/25,
  25/75, 40/30/30, 50/25/25, 25/25/50, 25/50/25. The numeric Columns
  field remains for setting the matching column count (Universal Editor
  has no supported API to auto-insert columns from a select change, so
  count stays author-driven — documented in the field description).
- columns.css applies per-ratio flex-basis widths at >=900px; equal
  (no class) keeps the existing behavior; mobile stacks.
- Removed blocks/columns-control and its importer parser; merkle-now
  featured section now imports as core Columns with the layout variant
  (layout-40-30-30 + layout-25-25-50). Regenerated content + JCR.

Verified all six ratios compute correct widths in preview.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-merkle-now.report.xlsx
+++ b/tools/importer/reports/import-merkle-now.report.xlsx
@@ -64,7 +64,7 @@
     <t>en/merkle-now.report.json</t>
   </si>
   <si>
-    <t>["columns-control"]</t>
+    <t>["columns"]</t>
   </si>
   <si>
     <t>en/merkle-now</t>
@@ -73,7 +73,7 @@
     <t>merkle-now</t>
   </si>
   <si>
-    <t>2026-09-17T06:39:57.072Z</t>
+    <t>2026-09-17T07:51:47.754Z</t>
   </si>
   <si>
     <t>Merkle Now: Thought Leadership, Culture &amp; Resources</t>

</xml_diff>